<commit_message>
Update data workbook: list tied domains in Balance, add domain scores of every analysed record, partial orders and dominance relations of each scenario, and the scenario summary
</commit_message>
<xml_diff>
--- a/searo-dht-data 19102026.xlsx
+++ b/searo-dht-data 19102026.xlsx
@@ -16,9 +16,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity indices" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Partial order heights" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mutual ranking prob" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bangladesh change" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity scenarios" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dominance relations" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mutual ranking prob" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bangladesh change" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity scenarios" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -437,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -509,11 +510,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Domain scores of the 6 primary records (mean of scored core indicators)</t>
+          <t>Domain scores of every analysed record, primary, change analysis and sensitivity (mean of scored core indicators)</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">
@@ -569,7 +570,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Domain balance metrics and the adjusted Mazziotta-Pareto index</t>
+          <t>Domain balance metrics and the adjusted Mazziotta-Pareto index (tied domains separated by /)</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -584,83 +585,98 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Average height and position range in the partial order</t>
+          <t>Average height and position range in the partial order of each scenario</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Mutual ranking prob</t>
+          <t>Dominance relations</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Mutual ranking probabilities in the partial order</t>
+          <t>Dominance relations of each scenario, with the cover relations drawn in the Hasse diagrams</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Bangladesh change</t>
+          <t>Mutual ranking prob</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Item phases of Bangladesh in 2023, 2024 and 2026</t>
+          <t>Mutual ranking probabilities in the partial order</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>31</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>Bangladesh change</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Item phases of Bangladesh in 2023, 2024 and 2026</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>Sensitivity scenarios</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Summary of the primary and sensitivity simulations</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Summary of the primary and sensitivity scenarios</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="14"/>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Global Digital Health Monitor public application programming interface, retrieved 19 October 2026</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>https://monitor.digitalhealthmonitor.org</t>
-        </is>
-      </c>
-    </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Global Digital Health Monitor public application programming interface, retrieved 19 October 2026</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>https://monitor.digitalhealthmonitor.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>Scope</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Aggregated country-level records only. No individual-level or restricted data.</t>
         </is>
@@ -672,6 +688,428 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="41" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="37" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Dominating country</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Dominated country</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Cover relation in the Hasse diagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Primary analysis</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Bangladesh</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="D2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Primary analysis</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="D3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Primary analysis</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Sri Lanka</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="D4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Primary analysis</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Myanmar</t>
+        </is>
+      </c>
+      <c r="D5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Primary analysis</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="D6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Bhutan and Maldives added</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Bangladesh</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Maldives</t>
+        </is>
+      </c>
+      <c r="D7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Bhutan and Maldives added</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Bangladesh</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="D8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Bhutan and Maldives added</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Bhutan</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Maldives</t>
+        </is>
+      </c>
+      <c r="D9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Bhutan and Maldives added</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Maldives</t>
+        </is>
+      </c>
+      <c r="D10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Bhutan and Maldives added</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="D11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Bhutan and Maldives added</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Sri Lanka</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="D12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Bhutan and Maldives added</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Maldives</t>
+        </is>
+      </c>
+      <c r="D13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Bhutan and Maldives added</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Myanmar</t>
+        </is>
+      </c>
+      <c r="D14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Bhutan and Maldives added</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="D15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Bangladesh 2024 record in place of 2026</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Bangladesh</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="D16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Bangladesh 2024 record in place of 2026</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="D17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Bangladesh 2024 record in place of 2026</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Sri Lanka</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="D18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Bangladesh 2024 record in place of 2026</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Myanmar</t>
+        </is>
+      </c>
+      <c r="D19" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Bangladesh 2024 record in place of 2026</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="D20" t="b">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -863,7 +1301,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1698,24 +2136,28 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="28" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="41" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="35" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="23" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="30" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1726,175 +2168,243 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>label</t>
+          <t>Countries (n)</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>n_units</t>
+          <t>Base draws (n)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>n_base</t>
+          <t>Model evaluations (n)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>n_model_runs</t>
+          <t>Reference order reproduced (share)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>mean_rank_shift_mean</t>
+          <t>Mean absolute rank shift</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>mean_rank_shift_p95</t>
+          <t>Largest total-order index, factor</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>share_runs_reference_order</t>
+          <t>Largest total-order index, value</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>share_runs_with_tied_ranks</t>
+          <t>Comparable pairs (n)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Pairs (n)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Linear extensions (n)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Indonesia phase retained (share)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Nepal phase retained (share)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>primary</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>primary</t>
-        </is>
+          <t>Primary analysis</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>6</v>
       </c>
       <c r="C2" t="n">
-        <v>6</v>
+        <v>65536</v>
       </c>
       <c r="D2" t="n">
-        <v>65536</v>
+        <v>458752</v>
       </c>
       <c r="E2" t="n">
-        <v>458752</v>
+        <v>0.88873291015625</v>
       </c>
       <c r="F2" t="n">
         <v>0.03814188639322916</v>
       </c>
-      <c r="G2" t="n">
-        <v>0.3333333333333333</v>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Domain weights</t>
+        </is>
       </c>
       <c r="H2" t="n">
-        <v>0.88873291015625</v>
+        <v>0.8326038473678833</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="J2" t="n">
+        <v>15</v>
+      </c>
+      <c r="K2" t="n">
+        <v>84</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.6136322021484375</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.3710784912109375</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>sens_bhutan_maldives</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>with_bhutan_maldives</t>
-        </is>
+          <t>Bhutan and Maldives added</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>8</v>
       </c>
       <c r="C3" t="n">
-        <v>8</v>
+        <v>65536</v>
       </c>
       <c r="D3" t="n">
-        <v>65536</v>
+        <v>458752</v>
       </c>
       <c r="E3" t="n">
-        <v>458752</v>
+        <v>0.4317092895507812</v>
       </c>
       <c r="F3" t="n">
         <v>0.1734714508056641</v>
       </c>
-      <c r="G3" t="n">
-        <v>0.5</v>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Aggregation level</t>
+        </is>
       </c>
       <c r="H3" t="n">
-        <v>0.4317092895507812</v>
+        <v>0.5958852062650118</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>9</v>
+      </c>
+      <c r="J3" t="n">
+        <v>28</v>
+      </c>
+      <c r="K3" t="n">
+        <v>1464</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.6118927001953125</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.3701705932617187</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>sens_bgd2024</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>bangladesh_2024</t>
-        </is>
+          <t>Bangladesh 2024 record in place of 2026</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>6</v>
       </c>
       <c r="C4" t="n">
-        <v>6</v>
+        <v>65536</v>
       </c>
       <c r="D4" t="n">
-        <v>65536</v>
+        <v>458752</v>
       </c>
       <c r="E4" t="n">
-        <v>458752</v>
+        <v>0.6555709838867188</v>
       </c>
       <c r="F4" t="n">
         <v>0.1245803833007812</v>
       </c>
-      <c r="G4" t="n">
-        <v>0.3333333333333333</v>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Aggregation level</t>
+        </is>
       </c>
       <c r="H4" t="n">
-        <v>0.6555709838867188</v>
+        <v>0.5013692311924048</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="J4" t="n">
+        <v>15</v>
+      </c>
+      <c r="K4" t="n">
+        <v>84</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.6103363037109375</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.3690643310546875</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>sens_dirichlet</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>dirichlet_weights</t>
-        </is>
+          <t>Unrestricted domain weights</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>6</v>
       </c>
       <c r="C5" t="n">
-        <v>6</v>
+        <v>65536</v>
       </c>
       <c r="D5" t="n">
-        <v>65536</v>
+        <v>458752</v>
       </c>
       <c r="E5" t="n">
-        <v>458752</v>
+        <v>0.7020797729492188</v>
       </c>
       <c r="F5" t="n">
         <v>0.129791259765625</v>
       </c>
-      <c r="G5" t="n">
-        <v>0.6666666666666666</v>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Aggregation level</t>
+        </is>
       </c>
       <c r="H5" t="n">
-        <v>0.7020797729492188</v>
+        <v>0.6751303963080835</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="J5" t="n">
+        <v>15</v>
+      </c>
+      <c r="K5" t="n">
+        <v>84</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.5253067016601562</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.3424758911132812</v>
       </c>
     </row>
   </sheetData>
@@ -29198,13 +29708,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
     <col width="27" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
     <col width="36" customWidth="1" min="7" max="7"/>
@@ -29232,7 +29742,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>use</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -29282,12 +29792,14 @@
           <t>Bangladesh</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>2026</v>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>approved</t>
+          <t>Primary</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -29323,12 +29835,14 @@
           <t>Indonesia</t>
         </is>
       </c>
-      <c r="C3" t="n">
-        <v>2023</v>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>approved</t>
+          <t>Primary</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -29364,12 +29878,14 @@
           <t>Sri Lanka</t>
         </is>
       </c>
-      <c r="C4" t="n">
-        <v>2024</v>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>approved</t>
+          <t>Primary</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -29405,12 +29921,14 @@
           <t>Myanmar</t>
         </is>
       </c>
-      <c r="C5" t="n">
-        <v>2023</v>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>approved</t>
+          <t>Primary</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -29446,12 +29964,14 @@
           <t>Nepal</t>
         </is>
       </c>
-      <c r="C6" t="n">
-        <v>2023</v>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>approved</t>
+          <t>Primary</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -29487,12 +30007,14 @@
           <t>Thailand</t>
         </is>
       </c>
-      <c r="C7" t="n">
-        <v>2023</v>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>approved</t>
+          <t>Primary</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -29515,6 +30037,178 @@
       </c>
       <c r="K7" t="n">
         <v>4.4</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BGD</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Bangladesh</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Change analysis</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>5</v>
+      </c>
+      <c r="F8" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="H8" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J8" t="n">
+        <v>4</v>
+      </c>
+      <c r="K8" t="n">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BGD</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Bangladesh</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Change analysis</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>5</v>
+      </c>
+      <c r="F9" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="H9" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J9" t="n">
+        <v>4</v>
+      </c>
+      <c r="K9" t="n">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BTN</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Bhutan</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Sensitivity</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F10" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G10" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="I10" t="n">
+        <v>3</v>
+      </c>
+      <c r="J10" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" t="n">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>MDV</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Maldives</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Sensitivity</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>2.666666666666667</v>
+      </c>
+      <c r="F11" t="n">
+        <v>2</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" t="n">
+        <v>1.8</v>
       </c>
     </row>
   </sheetData>
@@ -30562,9 +31256,9 @@
     <col width="19" customWidth="1" min="9" max="9"/>
     <col width="19" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="60" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="36" customWidth="1" min="14" max="14"/>
+    <col width="60" customWidth="1" min="14" max="14"/>
     <col width="15" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
     <col width="11" customWidth="1" min="17" max="17"/>
@@ -30819,7 +31513,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Leadership and governance</t>
+          <t>Leadership and governance / Strategy and investment</t>
         </is>
       </c>
       <c r="M4" t="n">
@@ -30827,7 +31521,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Legislation, policy and compliance</t>
+          <t>Legislation, policy and compliance / Workforce / Standards and interoperability / Infrastructure</t>
         </is>
       </c>
       <c r="O4" t="n">
@@ -30880,7 +31574,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Legislation, policy and compliance</t>
+          <t>Legislation, policy and compliance / Workforce</t>
         </is>
       </c>
       <c r="M5" t="n">
@@ -30941,7 +31635,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Legislation, policy and compliance</t>
+          <t>Legislation, policy and compliance / Standards and interoperability</t>
         </is>
       </c>
       <c r="M6" t="n">
@@ -31010,7 +31704,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Leadership and governance</t>
+          <t>Leadership and governance / Legislation, policy and compliance</t>
         </is>
       </c>
       <c r="O7" t="n">
@@ -31034,7 +31728,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -31045,6 +31739,7 @@
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="41" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -31088,6 +31783,11 @@
           <t>n_incomparable</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>scenario</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -31118,6 +31818,11 @@
       <c r="H2" t="n">
         <v>4</v>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Primary analysis</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -31148,6 +31853,11 @@
       <c r="H3" t="n">
         <v>4</v>
       </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Primary analysis</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -31178,6 +31888,11 @@
       <c r="H4" t="n">
         <v>4</v>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Primary analysis</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -31208,6 +31923,11 @@
       <c r="H5" t="n">
         <v>4</v>
       </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Primary analysis</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -31238,6 +31958,11 @@
       <c r="H6" t="n">
         <v>1</v>
       </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Primary analysis</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -31267,6 +31992,501 @@
       </c>
       <c r="H7" t="n">
         <v>3</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Primary analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BGD</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Bangladesh</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>3.19672131147541</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>6</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>5</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Bhutan and Maldives added</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BTN</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Bhutan</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>3.549180327868852</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>7</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Bhutan and Maldives added</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>IDN</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>3.19672131147541</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="n">
+        <v>6</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>5</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Bhutan and Maldives added</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>LKA</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Sri Lanka</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>3.549180327868852</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" t="n">
+        <v>7</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>6</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Bhutan and Maldives added</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>MDV</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Maldives</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>7.098360655737705</v>
+      </c>
+      <c r="D12" t="n">
+        <v>5</v>
+      </c>
+      <c r="E12" t="n">
+        <v>8</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>4</v>
+      </c>
+      <c r="H12" t="n">
+        <v>3</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Bhutan and Maldives added</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>MMR</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Myanmar</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>5.770491803278689</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" t="n">
+        <v>8</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" t="n">
+        <v>6</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Bhutan and Maldives added</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>NPL</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>7.098360655737705</v>
+      </c>
+      <c r="D14" t="n">
+        <v>5</v>
+      </c>
+      <c r="E14" t="n">
+        <v>8</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H14" t="n">
+        <v>3</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Bhutan and Maldives added</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>THA</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>2.540983606557377</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="n">
+        <v>5</v>
+      </c>
+      <c r="F15" t="n">
+        <v>3</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>4</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Bhutan and Maldives added</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>BGD</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Bangladesh</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>2.857142857142857</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="n">
+        <v>5</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>4</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Bangladesh 2024 record in place of 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>IDN</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>2.857142857142857</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>5</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>4</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Bangladesh 2024 record in place of 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>LKA</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Sri Lanka</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>2.857142857142857</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="n">
+        <v>5</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
+        <v>4</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Bangladesh 2024 record in place of 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>MMR</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Myanmar</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>4.571428571428571</v>
+      </c>
+      <c r="D19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E19" t="n">
+        <v>6</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" t="n">
+        <v>4</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Bangladesh 2024 record in place of 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>NPL</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Nepal</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>5.714285714285714</v>
+      </c>
+      <c r="D20" t="n">
+        <v>5</v>
+      </c>
+      <c r="E20" t="n">
+        <v>6</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="n">
+        <v>4</v>
+      </c>
+      <c r="H20" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Bangladesh 2024 record in place of 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>THA</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>2.142857142857143</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" t="n">
+        <v>4</v>
+      </c>
+      <c r="F21" t="n">
+        <v>2</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="n">
+        <v>3</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Bangladesh 2024 record in place of 2026</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>